<commit_message>
061025 - udpated results week 6 text
</commit_message>
<xml_diff>
--- a/public/results/2025/2025 Weekly Stats - Week 6.xlsx
+++ b/public/results/2025/2025 Weekly Stats - Week 6.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mthutter/CODE/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4714B3AD-2552-AF4A-B5A0-C8EDCE75B67B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF34B3A3-5DA3-6146-B922-F1643D786C17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4240" yWindow="2240" windowWidth="29860" windowHeight="16420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4240" yWindow="2240" windowWidth="29860" windowHeight="16420" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="14" r:id="rId1"/>

</xml_diff>